<commit_message>
feat: Gün 2 tamamlandı - Zamanlayıcı, loglama, sağlamlaştırma ve Rakip B (webscraper.io) eklendi
</commit_message>
<xml_diff>
--- a/data/urunlerim.xlsx
+++ b/data/urunlerim.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -968,6 +968,216 @@
         <v>20</v>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>EL-001</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Lenovo IdeaTab (7 inç Android)</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>2550</v>
+      </c>
+      <c r="D27" t="n">
+        <v>1800</v>
+      </c>
+      <c r="E27" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>EL-002</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>IdeaTab A3500L</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>3100</v>
+      </c>
+      <c r="D28" t="n">
+        <v>2200</v>
+      </c>
+      <c r="E28" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>EL-003</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Acer Iconia (16GB Tablet)</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>3500</v>
+      </c>
+      <c r="D29" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E29" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>EL-004</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Iconia B1-730HD</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>3600</v>
+      </c>
+      <c r="D30" t="n">
+        <v>2600</v>
+      </c>
+      <c r="E30" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>EL-005</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Memo Pad HD 7</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>3650</v>
+      </c>
+      <c r="D31" t="n">
+        <v>2650</v>
+      </c>
+      <c r="E31" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>EL-006</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Asus MeMO Pad</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>3550</v>
+      </c>
+      <c r="D32" t="n">
+        <v>2550</v>
+      </c>
+      <c r="E32" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>EL-007</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Amazon Kindle</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>3750</v>
+      </c>
+      <c r="D33" t="n">
+        <v>2700</v>
+      </c>
+      <c r="E33" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>EL-008</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>IdeaTab A8-50</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>4400</v>
+      </c>
+      <c r="D34" t="n">
+        <v>3100</v>
+      </c>
+      <c r="E34" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>EL-009</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>iPad Mini Retina (Wi-Fi)</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>19200</v>
+      </c>
+      <c r="D35" t="n">
+        <v>14500</v>
+      </c>
+      <c r="E35" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>EL-010</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Apple iPad Air</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>21500</v>
+      </c>
+      <c r="D36" t="n">
+        <v>16000</v>
+      </c>
+      <c r="E36" t="n">
+        <v>20</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: Gün 1-2 denetimi - Eşleştirme tie-breaker, onay_bekliyor verileri ve kök script uyumluluğu
</commit_message>
<xml_diff>
--- a/data/urunlerim.xlsx
+++ b/data/urunlerim.xlsx
@@ -808,14 +808,14 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Mesa Selimovic - Death and the Dervish</t>
+          <t>Mesaerion: Best Science Hikayeleri 1800-1849</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>750</v>
+        <v>1550</v>
       </c>
       <c r="D19" t="n">
-        <v>500</v>
+        <v>1050</v>
       </c>
       <c r="E19" t="n">
         <v>20</v>
@@ -829,17 +829,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Frankenstein</t>
+          <t>Libertarian for Beginners Rehberi</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>1550</v>
+        <v>2100</v>
       </c>
       <c r="D20" t="n">
-        <v>1000</v>
+        <v>1450</v>
       </c>
       <c r="E20" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="21">
@@ -850,14 +850,14 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Forever and Forever</t>
+          <t>Only the Himalayas Gezi Kitabı</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1200</v>
+        <v>1850</v>
       </c>
       <c r="D21" t="n">
-        <v>800</v>
+        <v>1250</v>
       </c>
       <c r="E21" t="n">
         <v>20</v>
@@ -871,14 +871,14 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Emma</t>
+          <t>Foolproof Preserving Reçel Rehberi</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1350</v>
+        <v>1300</v>
       </c>
       <c r="D22" t="n">
-        <v>900</v>
+        <v>850</v>
       </c>
       <c r="E22" t="n">
         <v>20</v>
@@ -892,14 +892,14 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Alice in Wonderland</t>
+          <t>In Her Wake (Polisiye)</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>2250</v>
+        <v>550</v>
       </c>
       <c r="D23" t="n">
-        <v>1500</v>
+        <v>380</v>
       </c>
       <c r="E23" t="n">
         <v>20</v>
@@ -913,17 +913,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ajin: Demi-Human, Volume 1</t>
+          <t>How Music Works</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>1750</v>
+        <v>1520</v>
       </c>
       <c r="D24" t="n">
-        <v>1150</v>
+        <v>1050</v>
       </c>
       <c r="E24" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="25">
@@ -934,14 +934,14 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>A Spy's Alone</t>
+          <t>Chase Me (Paris Nights)</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>2050</v>
+        <v>1050</v>
       </c>
       <c r="D25" t="n">
-        <v>1350</v>
+        <v>700</v>
       </c>
       <c r="E25" t="n">
         <v>20</v>
@@ -955,14 +955,14 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>1,000 Places to See Before You Die</t>
+          <t>Black Dust</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>1100</v>
+        <v>1350</v>
       </c>
       <c r="D26" t="n">
-        <v>750</v>
+        <v>920</v>
       </c>
       <c r="E26" t="n">
         <v>20</v>

</xml_diff>